<commit_message>
Cierre formal de los Sprints 1, 2, 3 y 5: Definition of Done marcada y criterios de lo movido al Sprint 6
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Sprint Backlogs/SIGMA_Sprint_Backlog_S1.xlsx
+++ b/Fase 2/Evidencias Proyecto/Sprint Backlogs/SIGMA_Sprint_Backlog_S1.xlsx
@@ -16024,7 +16024,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -16064,7 +16064,7 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -16084,7 +16084,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -16104,7 +16104,7 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -16124,7 +16124,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -16144,10 +16144,11 @@
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="24">
       <c r="A16" s="27" t="inlineStr">
         <is>

</xml_diff>